<commit_message>
[fix] per_frame and per_video get same metric values
</commit_message>
<xml_diff>
--- a/_issue_track.xlsx
+++ b/_issue_track.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SyncData\paper2_main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EE4B377-3B62-4957-A90D-8E416F8DB426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{292BA7F9-4C0A-40C7-B0D9-CBA3FB144A68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17010" yWindow="-120" windowWidth="28110" windowHeight="16440" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="285" windowWidth="16440" windowHeight="28035" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Example Issue Tracking" sheetId="4" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="45">
   <si>
     <t xml:space="preserve">Any articles, templates, or information provided by Smartsheet on the website are for reference only. While we strive to keep the information up to date and correct, we make no representations or warranties of any kind, express or implied, about the completeness, accuracy, reliability, suitability, or availability with respect to the website or the information, articles, templates, or related graphics contained on the website. Any reliance you place on such information is therefore strictly at your own risk. </t>
   </si>
@@ -165,6 +165,21 @@
   </si>
   <si>
     <t>slow speed when drawing text for video visualization when using custom</t>
+  </si>
+  <si>
+    <t>2026.03.06</t>
+  </si>
+  <si>
+    <t>iss04</t>
+  </si>
+  <si>
+    <t>some labels in videos is INCORRECT (need to re-annotate)</t>
+  </si>
+  <si>
+    <t>iss05</t>
+  </si>
+  <si>
+    <t>current Code can not compared with external exp (results from cls or od models)</t>
   </si>
 </sst>
 </file>
@@ -595,7 +610,161 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="5" xr:uid="{C1547B1A-ACFD-7E4D-8269-7F11392CAD83}"/>
   </cellStyles>
-  <dxfs count="33">
+  <dxfs count="55">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFED2B38"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF3EB8EE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9966"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE54B1B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF3EB8EE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9966"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -831,6 +1000,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <colors>
     <mruColors>
+      <color rgb="FFED2B38"/>
+      <color rgb="FFFF9966"/>
       <color rgb="FFE54B1B"/>
       <color rgb="FF3EB8EE"/>
       <color rgb="FF00BD32"/>
@@ -1301,7 +1472,7 @@
         <v>36</v>
       </c>
       <c r="D5" s="48" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E5" s="48" t="s">
         <v>20</v>
@@ -1323,8 +1494,12 @@
     </row>
     <row r="6" spans="1:15" s="37" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="36"/>
-      <c r="B6" s="40"/>
-      <c r="C6" s="40"/>
+      <c r="B6" s="40" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="40" t="s">
+        <v>41</v>
+      </c>
       <c r="D6" s="48" t="s">
         <v>17</v>
       </c>
@@ -1332,9 +1507,11 @@
         <v>20</v>
       </c>
       <c r="F6" s="48" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
-      <c r="G6" s="39"/>
+      <c r="G6" s="39" t="s">
+        <v>42</v>
+      </c>
       <c r="H6" s="41"/>
       <c r="I6" s="36"/>
       <c r="J6" s="36"/>
@@ -1346,10 +1523,14 @@
     </row>
     <row r="7" spans="1:15" s="37" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="36"/>
-      <c r="B7" s="40"/>
-      <c r="C7" s="40"/>
+      <c r="B7" s="40" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="40" t="s">
+        <v>43</v>
+      </c>
       <c r="D7" s="48" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E7" s="48" t="s">
         <v>20</v>
@@ -1357,7 +1538,9 @@
       <c r="F7" s="48" t="s">
         <v>24</v>
       </c>
-      <c r="G7" s="39"/>
+      <c r="G7" s="39" t="s">
+        <v>44</v>
+      </c>
       <c r="H7" s="41"/>
       <c r="I7" s="36"/>
       <c r="J7" s="36"/>
@@ -6418,41 +6601,41 @@
   <autoFilter ref="C2:H2" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <phoneticPr fontId="17" type="noConversion"/>
   <conditionalFormatting sqref="D3:F27">
-    <cfRule type="containsText" dxfId="32" priority="9" operator="containsText" text="Closed">
+    <cfRule type="containsText" dxfId="10" priority="9" operator="containsText" text="Closed">
       <formula>NOT(ISERROR(SEARCH("Closed",D3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="31" priority="10" operator="containsText" text="In Progress">
+    <cfRule type="containsText" dxfId="9" priority="10" operator="containsText" text="In Progress">
       <formula>NOT(ISERROR(SEARCH("In Progress",D3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="30" priority="11" operator="containsText" text="Open">
+    <cfRule type="containsText" dxfId="8" priority="11" operator="containsText" text="Open">
       <formula>NOT(ISERROR(SEARCH("Open",D3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E3:E27">
-    <cfRule type="containsText" dxfId="29" priority="5" operator="containsText" text="Request">
+    <cfRule type="containsText" dxfId="7" priority="5" operator="containsText" text="Request">
       <formula>NOT(ISERROR(SEARCH("Request",E3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="28" priority="6" operator="containsText" text="Task">
+    <cfRule type="containsText" dxfId="6" priority="6" operator="containsText" text="Task">
       <formula>NOT(ISERROR(SEARCH("Task",E3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="27" priority="7" operator="containsText" text="Feature">
+    <cfRule type="containsText" dxfId="5" priority="7" operator="containsText" text="Feature">
       <formula>NOT(ISERROR(SEARCH("Feature",E3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="26" priority="8" operator="containsText" text="Bug">
+    <cfRule type="containsText" dxfId="4" priority="8" operator="containsText" text="Bug">
       <formula>NOT(ISERROR(SEARCH("Bug",E3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:F27">
-    <cfRule type="containsText" dxfId="25" priority="1" operator="containsText" text="Critical">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Critical">
       <formula>NOT(ISERROR(SEARCH("Critical",F3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="24" priority="2" operator="containsText" text="High">
+    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="High">
       <formula>NOT(ISERROR(SEARCH("High",F3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="23" priority="3" operator="containsText" text="Medium">
+    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Medium">
       <formula>NOT(ISERROR(SEARCH("Medium",F3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="22" priority="4" operator="containsText" text="Low">
+    <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="Low">
       <formula>NOT(ISERROR(SEARCH("Low",F3)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13470,41 +13653,41 @@
     <mergeCell ref="D5:E5"/>
   </mergeCells>
   <conditionalFormatting sqref="C8:C32">
-    <cfRule type="containsText" dxfId="21" priority="9" operator="containsText" text="Closed">
+    <cfRule type="containsText" dxfId="54" priority="9" operator="containsText" text="Closed">
       <formula>NOT(ISERROR(SEARCH("Closed",C8)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="20" priority="10" operator="containsText" text="In Progress">
+    <cfRule type="containsText" dxfId="53" priority="10" operator="containsText" text="In Progress">
       <formula>NOT(ISERROR(SEARCH("In Progress",C8)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="19" priority="11" operator="containsText" text="Open">
+    <cfRule type="containsText" dxfId="52" priority="11" operator="containsText" text="Open">
       <formula>NOT(ISERROR(SEARCH("Open",C8)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8:E32">
-    <cfRule type="containsText" dxfId="18" priority="5" operator="containsText" text="Request">
+    <cfRule type="containsText" dxfId="51" priority="5" operator="containsText" text="Request">
       <formula>NOT(ISERROR(SEARCH("Request",E8)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="17" priority="6" operator="containsText" text="Task">
+    <cfRule type="containsText" dxfId="50" priority="6" operator="containsText" text="Task">
       <formula>NOT(ISERROR(SEARCH("Task",E8)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="16" priority="7" operator="containsText" text="Feature">
+    <cfRule type="containsText" dxfId="49" priority="7" operator="containsText" text="Feature">
       <formula>NOT(ISERROR(SEARCH("Feature",E8)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="8" operator="containsText" text="Bug">
+    <cfRule type="containsText" dxfId="48" priority="8" operator="containsText" text="Bug">
       <formula>NOT(ISERROR(SEARCH("Bug",E8)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F8:F32">
-    <cfRule type="containsText" dxfId="14" priority="1" operator="containsText" text="Critical">
+    <cfRule type="containsText" dxfId="47" priority="1" operator="containsText" text="Critical">
       <formula>NOT(ISERROR(SEARCH("Critical",F8)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="High">
+    <cfRule type="containsText" dxfId="46" priority="2" operator="containsText" text="High">
       <formula>NOT(ISERROR(SEARCH("High",F8)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="3" operator="containsText" text="Medium">
+    <cfRule type="containsText" dxfId="45" priority="3" operator="containsText" text="Medium">
       <formula>NOT(ISERROR(SEARCH("Medium",F8)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="11" priority="4" operator="containsText" text="Low">
+    <cfRule type="containsText" dxfId="44" priority="4" operator="containsText" text="Low">
       <formula>NOT(ISERROR(SEARCH("Low",F8)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13627,41 +13810,41 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B4:B6">
-    <cfRule type="containsText" dxfId="10" priority="9" operator="containsText" text="Closed">
+    <cfRule type="containsText" dxfId="43" priority="9" operator="containsText" text="Closed">
       <formula>NOT(ISERROR(SEARCH("Closed",B4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="10" operator="containsText" text="In Progress">
+    <cfRule type="containsText" dxfId="42" priority="10" operator="containsText" text="In Progress">
       <formula>NOT(ISERROR(SEARCH("In Progress",B4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="11" operator="containsText" text="Open">
+    <cfRule type="containsText" dxfId="41" priority="11" operator="containsText" text="Open">
       <formula>NOT(ISERROR(SEARCH("Open",B4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:C7">
-    <cfRule type="containsText" dxfId="7" priority="5" operator="containsText" text="Request">
+    <cfRule type="containsText" dxfId="40" priority="5" operator="containsText" text="Request">
       <formula>NOT(ISERROR(SEARCH("Request",C4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="6" operator="containsText" text="Task">
+    <cfRule type="containsText" dxfId="39" priority="6" operator="containsText" text="Task">
       <formula>NOT(ISERROR(SEARCH("Task",C4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="7" operator="containsText" text="Feature">
+    <cfRule type="containsText" dxfId="38" priority="7" operator="containsText" text="Feature">
       <formula>NOT(ISERROR(SEARCH("Feature",C4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="8" operator="containsText" text="Bug">
+    <cfRule type="containsText" dxfId="37" priority="8" operator="containsText" text="Bug">
       <formula>NOT(ISERROR(SEARCH("Bug",C4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D4:D7">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Critical">
+    <cfRule type="containsText" dxfId="36" priority="1" operator="containsText" text="Critical">
       <formula>NOT(ISERROR(SEARCH("Critical",D4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="High">
+    <cfRule type="containsText" dxfId="35" priority="2" operator="containsText" text="High">
       <formula>NOT(ISERROR(SEARCH("High",D4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="Medium">
+    <cfRule type="containsText" dxfId="34" priority="3" operator="containsText" text="Medium">
       <formula>NOT(ISERROR(SEARCH("Medium",D4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="4" operator="containsText" text="Low">
+    <cfRule type="containsText" dxfId="33" priority="4" operator="containsText" text="Low">
       <formula>NOT(ISERROR(SEARCH("Low",D4)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[refactor] re-organize folder structure
</commit_message>
<xml_diff>
--- a/_issue_track.xlsx
+++ b/_issue_track.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SyncData\paper2_main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C844106-1A86-40B4-8F11-B2D08B58FBA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E82A4C3-9D81-4BA9-8797-3B4EA3710FC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17010" yWindow="-120" windowWidth="28110" windowHeight="16440" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="48">
   <si>
     <t xml:space="preserve">Any articles, templates, or information provided by Smartsheet on the website are for reference only. While we strive to keep the information up to date and correct, we make no representations or warranties of any kind, express or implied, about the completeness, accuracy, reliability, suitability, or availability with respect to the website or the information, articles, templates, or related graphics contained on the website. Any reliance you place on such information is therefore strictly at your own risk. </t>
   </si>
@@ -152,9 +152,6 @@
     <t>iss02</t>
   </si>
   <si>
-    <t>fixed</t>
-  </si>
-  <si>
     <t>iss03</t>
   </si>
   <si>
@@ -183,6 +180,15 @@
   </si>
   <si>
     <t>done (ignore using draw by font, but use native opencv2 text draw)</t>
+  </si>
+  <si>
+    <t>2026.03.09</t>
+  </si>
+  <si>
+    <t>iss06</t>
+  </si>
+  <si>
+    <t>incorrect per-frame and per-video resutls (between test code and exp metric calc code)</t>
   </si>
 </sst>
 </file>
@@ -313,7 +319,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FFFF0000"/>
       <name val="Roboto"/>
     </font>
   </fonts>
@@ -594,15 +599,15 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="7" fontId="18" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="7" fontId="18" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1270,8 +1275,8 @@
       <c r="G3" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="H3" s="49" t="s">
-        <v>35</v>
+      <c r="H3" s="51" t="s">
+        <v>37</v>
       </c>
       <c r="I3" s="36"/>
       <c r="J3" s="36"/>
@@ -1299,10 +1304,10 @@
         <v>24</v>
       </c>
       <c r="G4" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="H4" s="41" t="s">
         <v>37</v>
-      </c>
-      <c r="H4" s="41" t="s">
-        <v>38</v>
       </c>
       <c r="I4" s="36"/>
       <c r="J4" s="36"/>
@@ -1318,7 +1323,7 @@
         <v>33</v>
       </c>
       <c r="C5" s="40" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D5" s="48" t="s">
         <v>19</v>
@@ -1330,10 +1335,10 @@
         <v>24</v>
       </c>
       <c r="G5" s="39" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H5" s="41" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I5" s="36"/>
       <c r="J5" s="36"/>
@@ -1346,24 +1351,26 @@
     <row r="6" spans="1:15" s="37" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="36"/>
       <c r="B6" s="40" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C6" s="40" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D6" s="48" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E6" s="48" t="s">
         <v>20</v>
       </c>
       <c r="F6" s="48" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G6" s="39" t="s">
-        <v>42</v>
-      </c>
-      <c r="H6" s="41"/>
+        <v>43</v>
+      </c>
+      <c r="H6" s="41" t="s">
+        <v>37</v>
+      </c>
       <c r="I6" s="36"/>
       <c r="J6" s="36"/>
       <c r="K6" s="36"/>
@@ -1372,13 +1379,13 @@
       <c r="N6" s="36"/>
       <c r="O6" s="36"/>
     </row>
-    <row r="7" spans="1:15" s="37" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" s="37" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="36"/>
       <c r="B7" s="40" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C7" s="40" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D7" s="48" t="s">
         <v>19</v>
@@ -1387,13 +1394,13 @@
         <v>20</v>
       </c>
       <c r="F7" s="48" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G7" s="39" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H7" s="41" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I7" s="36"/>
       <c r="J7" s="36"/>
@@ -1403,10 +1410,14 @@
       <c r="N7" s="36"/>
       <c r="O7" s="36"/>
     </row>
-    <row r="8" spans="1:15" s="37" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" s="37" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="36"/>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
+      <c r="B8" s="40" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="40" t="s">
+        <v>40</v>
+      </c>
       <c r="D8" s="48" t="s">
         <v>17</v>
       </c>
@@ -1414,9 +1425,11 @@
         <v>20</v>
       </c>
       <c r="F8" s="48" t="s">
-        <v>24</v>
-      </c>
-      <c r="G8" s="39"/>
+        <v>27</v>
+      </c>
+      <c r="G8" s="39" t="s">
+        <v>41</v>
+      </c>
       <c r="H8" s="41"/>
       <c r="I8" s="36"/>
       <c r="J8" s="36"/>
@@ -1426,7 +1439,7 @@
       <c r="N8" s="36"/>
       <c r="O8" s="36"/>
     </row>
-    <row r="9" spans="1:15" s="37" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" s="37" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="36"/>
       <c r="B9" s="40"/>
       <c r="C9" s="40"/>
@@ -6451,7 +6464,11 @@
       <c r="H710" s="44"/>
     </row>
   </sheetData>
-  <autoFilter ref="C2:H2" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="C2:H2" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C3:H27">
+      <sortCondition ref="D2"/>
+    </sortState>
+  </autoFilter>
   <phoneticPr fontId="17" type="noConversion"/>
   <conditionalFormatting sqref="D3:F27">
     <cfRule type="containsText" dxfId="32" priority="9" operator="containsText" text="Closed">
@@ -6560,12 +6577,12 @@
       <c r="L1" s="14"/>
     </row>
     <row r="2" spans="1:19" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="50" t="s">
+      <c r="B2" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="50"/>
-      <c r="D2" s="51"/>
-      <c r="E2" s="51"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
       <c r="F2" s="21"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
@@ -6577,12 +6594,12 @@
       <c r="S2" s="2"/>
     </row>
     <row r="3" spans="1:19" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="50" t="s">
+      <c r="B3" s="49" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="50"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="51"/>
+      <c r="C3" s="49"/>
+      <c r="D3" s="50"/>
+      <c r="E3" s="50"/>
       <c r="F3" s="21"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
@@ -6594,12 +6611,12 @@
       <c r="S3" s="2"/>
     </row>
     <row r="4" spans="1:19" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="50" t="s">
+      <c r="B4" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="50"/>
-      <c r="D4" s="51"/>
-      <c r="E4" s="51"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="50"/>
+      <c r="E4" s="50"/>
       <c r="F4" s="21"/>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
@@ -6611,12 +6628,12 @@
       <c r="S4" s="2"/>
     </row>
     <row r="5" spans="1:19" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="50" t="s">
+      <c r="B5" s="49" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="50"/>
-      <c r="D5" s="51"/>
-      <c r="E5" s="51"/>
+      <c r="C5" s="49"/>
+      <c r="D5" s="50"/>
+      <c r="E5" s="50"/>
       <c r="F5" s="21"/>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>

</xml_diff>